<commit_message>
updated message and output variables; with corresponding updates in validation sheet
</commit_message>
<xml_diff>
--- a/rules/CORE-000029/negative/01/data/unit-test-coreid-CG0661-negative.xlsx
+++ b/rules/CORE-000029/negative/01/data/unit-test-coreid-CG0661-negative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000029\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BA22F3-0611-42D7-95A4-D7D523A4CFB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{472D9A76-AE08-4618-8987-18F358F4E885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="108">
   <si>
     <t>Product</t>
   </si>
@@ -340,6 +340,15 @@
   </si>
   <si>
     <t>2</t>
+  </si>
+  <si>
+    <t>LBTPT</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
+  </si>
+  <si>
+    <t>FTTPT</t>
   </si>
 </sst>
 </file>
@@ -1274,7 +1283,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -1324,10 +1333,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1336,10 +1345,50 @@
         <v>1</v>
       </c>
       <c r="E3" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F4" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>